<commit_message>
added execel reader data provider
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/phoenixTestData.xlsx
+++ b/src/test/resources/testData/phoenixTestData.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="CreateJobTestData" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="43">
   <si>
     <t>username</t>
   </si>
@@ -34,6 +34,117 @@
   </si>
   <si>
     <t>praveen@123</t>
+  </si>
+  <si>
+    <t>mst_service_location_id</t>
+  </si>
+  <si>
+    <t>mst_platform_id</t>
+  </si>
+  <si>
+    <t>mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t>mst_oem_id</t>
+  </si>
+  <si>
+    <t>customer__first_name</t>
+  </si>
+  <si>
+    <t>customer__last_name</t>
+  </si>
+  <si>
+    <t>customer__mobile_number</t>
+  </si>
+  <si>
+    <t>customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t>customer__email_id</t>
+  </si>
+  <si>
+    <t>customer__email_id_alt</t>
+  </si>
+  <si>
+    <t>customer_address__flat_number</t>
+  </si>
+  <si>
+    <t>customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t>customer_address__street_name</t>
+  </si>
+  <si>
+    <t>customer_address__landmark</t>
+  </si>
+  <si>
+    <t>customer_address__area</t>
+  </si>
+  <si>
+    <t>customer_address__state</t>
+  </si>
+  <si>
+    <t>customer_address__country</t>
+  </si>
+  <si>
+    <t>customer_address__pincode</t>
+  </si>
+  <si>
+    <t>customer_product__dop</t>
+  </si>
+  <si>
+    <t>customer_product__serial_number</t>
+  </si>
+  <si>
+    <t>customer_product__imei1</t>
+  </si>
+  <si>
+    <t>customer_product__imei2</t>
+  </si>
+  <si>
+    <t>customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t>customer_product__product_id</t>
+  </si>
+  <si>
+    <t>customer_product__popurl</t>
+  </si>
+  <si>
+    <t>problems__id</t>
+  </si>
+  <si>
+    <t>problems__remark</t>
+  </si>
+  <si>
+    <t>Praveen</t>
+  </si>
+  <si>
+    <t>Sharma</t>
+  </si>
+  <si>
+    <t>psagra13@gmail.com</t>
+  </si>
+  <si>
+    <t>xyz@gmail.com</t>
+  </si>
+  <si>
+    <t>GaneshVihar</t>
+  </si>
+  <si>
+    <t>Noida</t>
+  </si>
+  <si>
+    <t>Assam</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>2026-02-16T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t>Poor Battery</t>
   </si>
 </sst>
 </file>
@@ -64,12 +175,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -80,9 +206,15 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -426,10 +558,898 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="28.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="34.88671875" style="2" customWidth="1"/>
+    <col min="21" max="22" width="22.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="30.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="23.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12" style="2" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.88671875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H2" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="2">
+        <v>22</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R2" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T2" s="3" t="str">
+        <f ca="1">TEXT(TODAY(),"yyMMdd") &amp; TEXT(ROW()-2,"0000000000")</f>
+        <v>2603290000000000</v>
+      </c>
+      <c r="U2" s="3" t="str">
+        <f ca="1">T2</f>
+        <v>2603290000000000</v>
+      </c>
+      <c r="V2" s="3" t="str">
+        <f ca="1">U2</f>
+        <v>2603290000000000</v>
+      </c>
+      <c r="W2" s="2">
+        <v>1</v>
+      </c>
+      <c r="X2" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z2" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27">
+      <c r="A3" s="2">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H3" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="2">
+        <v>22</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R3" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T3" s="3" t="str">
+        <f t="shared" ref="T3:T10" ca="1" si="0">TEXT(TODAY(),"yyMMdd") &amp; TEXT(ROW()-2,"0000000000")</f>
+        <v>2603290000000001</v>
+      </c>
+      <c r="U3" s="3" t="str">
+        <f t="shared" ref="U3:V10" ca="1" si="1">T3</f>
+        <v>2603290000000001</v>
+      </c>
+      <c r="V3" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000001</v>
+      </c>
+      <c r="W3" s="2">
+        <v>1</v>
+      </c>
+      <c r="X3" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z3" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27">
+      <c r="A4" s="2">
+        <v>0</v>
+      </c>
+      <c r="B4" s="2">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H4" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="2">
+        <v>22</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T4" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2603290000000002</v>
+      </c>
+      <c r="U4" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000002</v>
+      </c>
+      <c r="V4" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000002</v>
+      </c>
+      <c r="W4" s="2">
+        <v>1</v>
+      </c>
+      <c r="X4" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z4" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA4" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27">
+      <c r="A5" s="2">
+        <v>0</v>
+      </c>
+      <c r="B5" s="2">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H5" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="2">
+        <v>22</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R5" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T5" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2603290000000003</v>
+      </c>
+      <c r="U5" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000003</v>
+      </c>
+      <c r="V5" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000003</v>
+      </c>
+      <c r="W5" s="2">
+        <v>1</v>
+      </c>
+      <c r="X5" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z5" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA5" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27">
+      <c r="A6" s="2">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H6" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" s="2">
+        <v>22</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R6" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T6" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2603290000000004</v>
+      </c>
+      <c r="U6" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000004</v>
+      </c>
+      <c r="V6" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000004</v>
+      </c>
+      <c r="W6" s="2">
+        <v>1</v>
+      </c>
+      <c r="X6" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z6" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA6" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27">
+      <c r="A7" s="2">
+        <v>0</v>
+      </c>
+      <c r="B7" s="2">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H7" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="2">
+        <v>22</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R7" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T7" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2603290000000005</v>
+      </c>
+      <c r="U7" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000005</v>
+      </c>
+      <c r="V7" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000005</v>
+      </c>
+      <c r="W7" s="2">
+        <v>1</v>
+      </c>
+      <c r="X7" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z7" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA7" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27">
+      <c r="A8" s="2">
+        <v>0</v>
+      </c>
+      <c r="B8" s="2">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H8" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="2">
+        <v>22</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R8" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T8" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2603290000000006</v>
+      </c>
+      <c r="U8" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000006</v>
+      </c>
+      <c r="V8" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000006</v>
+      </c>
+      <c r="W8" s="2">
+        <v>1</v>
+      </c>
+      <c r="X8" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z8" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA8" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27">
+      <c r="A9" s="2">
+        <v>0</v>
+      </c>
+      <c r="B9" s="2">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H9" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="2">
+        <v>22</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R9" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T9" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2603290000000007</v>
+      </c>
+      <c r="U9" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000007</v>
+      </c>
+      <c r="V9" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000007</v>
+      </c>
+      <c r="W9" s="2">
+        <v>1</v>
+      </c>
+      <c r="X9" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z9" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27">
+      <c r="A10" s="2">
+        <v>0</v>
+      </c>
+      <c r="B10" s="2">
+        <v>2</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="2">
+        <v>9990036806</v>
+      </c>
+      <c r="H10" s="2">
+        <v>9761759333</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="2">
+        <v>22</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R10" s="2">
+        <v>201301</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T10" s="3" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>2603290000000008</v>
+      </c>
+      <c r="U10" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000008</v>
+      </c>
+      <c r="V10" s="3" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>2603290000000008</v>
+      </c>
+      <c r="W10" s="2">
+        <v>1</v>
+      </c>
+      <c r="X10" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z10" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA10" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>